<commit_message>
Auto update claims data - Thu 08/06/2026 19:35:37.52
</commit_message>
<xml_diff>
--- a/الشركة العربية الأوروبية للتأمين.xlsx
+++ b/الشركة العربية الأوروبية للتأمين.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pharmacy_Operations\Insurance_Accounts\Insurance_Claims\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF96D667-7078-4EBE-9698-065F933CD984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84FA6145-CE80-4A37-B0AC-2D5BD3D6ED0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EE0FC3C9-C345-45F5-AA63-81B16FD29943}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="33">
   <si>
     <t>الرقم</t>
   </si>
@@ -126,6 +126,15 @@
   </si>
   <si>
     <t>محمد السعيدات</t>
+  </si>
+  <si>
+    <t>سارا رسمي السعيدات</t>
+  </si>
+  <si>
+    <t>ابراهيم جمعه زنون</t>
+  </si>
+  <si>
+    <t>قاسم دخيل الله القواسمه</t>
   </si>
 </sst>
 </file>
@@ -187,16 +196,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD29ECF-A88D-43BD-A0BB-A219CBC2F6D8}">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.5" bestFit="1" customWidth="1"/>
@@ -652,11 +658,11 @@
         <v>17.032</v>
       </c>
       <c r="J3" s="5">
-        <f t="shared" ref="J3:J43" si="0">G3*0.94-H3</f>
+        <f t="shared" ref="J3:J55" si="0">G3*0.94-H3</f>
         <v>15.7546</v>
       </c>
       <c r="L3" s="5">
-        <f t="shared" ref="L3:L43" si="1">J3-K3</f>
+        <f t="shared" ref="L3:L55" si="1">J3-K3</f>
         <v>15.7546</v>
       </c>
     </row>
@@ -2148,151 +2154,459 @@
       </c>
     </row>
     <row r="44" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A44" s="7">
+      <c r="A44" s="2">
         <v>1</v>
       </c>
-      <c r="B44" s="7">
+      <c r="B44" s="2">
         <v>780002702</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D44" s="7">
+      <c r="D44" s="2">
         <v>22</v>
       </c>
-      <c r="E44" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F44" s="8">
+      <c r="E44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" s="3">
         <v>46178</v>
       </c>
-      <c r="G44" s="7">
+      <c r="G44" s="2">
         <v>40.26</v>
       </c>
-      <c r="H44" s="7">
+      <c r="H44" s="2">
         <v>4.0259999999999998</v>
       </c>
-      <c r="I44" s="7">
+      <c r="I44" s="2">
         <v>36.234000000000002</v>
       </c>
-      <c r="J44" s="6"/>
-      <c r="K44" s="6"/>
-      <c r="L44" s="6"/>
-    </row>
-    <row r="45" spans="1:12" s="6" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45" s="7">
+      <c r="J44" s="5">
+        <f t="shared" si="0"/>
+        <v>33.818399999999997</v>
+      </c>
+      <c r="K44"/>
+      <c r="L44" s="5">
+        <f t="shared" si="1"/>
+        <v>33.818399999999997</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A45" s="2">
         <v>1</v>
       </c>
-      <c r="B45" s="7">
+      <c r="B45" s="2">
         <v>268583</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D45" s="7">
+      <c r="D45" s="2">
         <v>803447696</v>
       </c>
-      <c r="E45" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F45" s="8">
+      <c r="E45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F45" s="3">
         <v>45903</v>
       </c>
-      <c r="G45" s="7">
+      <c r="G45" s="2">
         <v>14.067</v>
       </c>
-      <c r="H45" s="7">
+      <c r="H45" s="2">
         <v>1.407</v>
       </c>
-      <c r="I45" s="7">
+      <c r="I45" s="2">
         <v>12.66</v>
       </c>
-    </row>
-    <row r="46" spans="1:12" s="6" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="7">
+      <c r="J45" s="5">
+        <f t="shared" si="0"/>
+        <v>11.81598</v>
+      </c>
+      <c r="K45"/>
+      <c r="L45" s="5">
+        <f t="shared" si="1"/>
+        <v>11.81598</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A46" s="2">
         <v>2</v>
       </c>
-      <c r="B46" s="7">
+      <c r="B46" s="2">
         <v>62004401</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="C46" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D46" s="7">
+      <c r="D46" s="2">
         <v>12610269342</v>
       </c>
-      <c r="E46" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F46" s="8">
+      <c r="E46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" s="3">
         <v>46140</v>
       </c>
-      <c r="G46" s="7">
+      <c r="G46" s="2">
         <v>12.5</v>
       </c>
-      <c r="H46" s="7">
+      <c r="H46" s="2">
         <v>1.925</v>
       </c>
-      <c r="I46" s="7">
+      <c r="I46" s="2">
         <v>10.574999999999999</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" s="6" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A47" s="7">
+      <c r="J46" s="5">
+        <f t="shared" si="0"/>
+        <v>9.8249999999999993</v>
+      </c>
+      <c r="K46"/>
+      <c r="L46" s="5">
+        <f t="shared" si="1"/>
+        <v>9.8249999999999993</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A47" s="2">
         <v>3</v>
       </c>
-      <c r="B47" s="7">
+      <c r="B47" s="2">
         <v>43001502</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="C47" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D47" s="7">
+      <c r="D47" s="2">
         <v>12610285384</v>
       </c>
-      <c r="E47" s="7" t="s">
+      <c r="E47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F47" s="8">
+      <c r="F47" s="3">
         <v>46164</v>
       </c>
-      <c r="G47" s="7">
+      <c r="G47" s="2">
         <v>12.5</v>
       </c>
-      <c r="H47" s="7">
+      <c r="H47" s="2">
         <v>1.25</v>
       </c>
-      <c r="I47" s="7">
+      <c r="I47" s="2">
         <v>11.25</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" s="6" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A48" s="7">
+      <c r="J47" s="5">
+        <f t="shared" si="0"/>
+        <v>10.5</v>
+      </c>
+      <c r="K47"/>
+      <c r="L47" s="5">
+        <f t="shared" si="1"/>
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A48" s="2">
         <v>4</v>
       </c>
-      <c r="B48" s="7">
+      <c r="B48" s="2">
         <v>50016401</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="C48" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D48" s="7">
+      <c r="D48" s="2">
         <v>12610292185</v>
       </c>
-      <c r="E48" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F48" s="8">
+      <c r="E48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F48" s="3">
         <v>46177</v>
       </c>
-      <c r="G48" s="7">
+      <c r="G48" s="2">
         <v>12.5</v>
       </c>
-      <c r="H48" s="7">
+      <c r="H48" s="2">
         <v>2.5</v>
       </c>
-      <c r="I48" s="7">
+      <c r="I48" s="2">
         <v>10</v>
+      </c>
+      <c r="J48" s="5">
+        <f t="shared" si="0"/>
+        <v>9.25</v>
+      </c>
+      <c r="K48"/>
+      <c r="L48" s="5">
+        <f t="shared" si="1"/>
+        <v>9.25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A49" s="2">
+        <v>1</v>
+      </c>
+      <c r="B49" s="2">
+        <v>780037005</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D49" s="2">
+        <v>12610309392</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F49" s="3">
+        <v>46207</v>
+      </c>
+      <c r="G49" s="2">
+        <v>44.66</v>
+      </c>
+      <c r="H49" s="2">
+        <v>4.4660000000000002</v>
+      </c>
+      <c r="I49" s="2">
+        <v>40.194000000000003</v>
+      </c>
+      <c r="J49" s="5">
+        <f t="shared" si="0"/>
+        <v>37.514399999999995</v>
+      </c>
+      <c r="K49"/>
+      <c r="L49" s="5">
+        <f t="shared" si="1"/>
+        <v>37.514399999999995</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A50" s="2">
+        <v>2</v>
+      </c>
+      <c r="B50" s="2">
+        <v>780037003</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D50" s="2">
+        <v>12610309395</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50" s="3">
+        <v>46207</v>
+      </c>
+      <c r="G50" s="2">
+        <v>54.41</v>
+      </c>
+      <c r="H50" s="2">
+        <v>5.4409999999999998</v>
+      </c>
+      <c r="I50" s="2">
+        <v>48.969000000000001</v>
+      </c>
+      <c r="J50" s="5">
+        <f t="shared" si="0"/>
+        <v>45.704399999999993</v>
+      </c>
+      <c r="K50"/>
+      <c r="L50" s="5">
+        <f t="shared" si="1"/>
+        <v>45.704399999999993</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A51" s="2">
+        <v>3</v>
+      </c>
+      <c r="B51" s="2">
+        <v>780002702</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" s="2">
+        <v>23</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F51" s="3">
+        <v>46209</v>
+      </c>
+      <c r="G51" s="2">
+        <v>40.26</v>
+      </c>
+      <c r="H51" s="2">
+        <v>4.0259999999999998</v>
+      </c>
+      <c r="I51" s="2">
+        <v>36.234000000000002</v>
+      </c>
+      <c r="J51" s="5">
+        <f t="shared" si="0"/>
+        <v>33.818399999999997</v>
+      </c>
+      <c r="K51"/>
+      <c r="L51" s="5">
+        <f t="shared" si="1"/>
+        <v>33.818399999999997</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A52" s="2">
+        <v>4</v>
+      </c>
+      <c r="B52" s="2">
+        <v>780037004</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D52" s="2">
+        <v>12610311180</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F52" s="3">
+        <v>46212</v>
+      </c>
+      <c r="G52" s="2">
+        <v>41.08</v>
+      </c>
+      <c r="H52" s="2">
+        <v>4.1079999999999997</v>
+      </c>
+      <c r="I52" s="2">
+        <v>36.972000000000001</v>
+      </c>
+      <c r="J52" s="5">
+        <f t="shared" si="0"/>
+        <v>34.507199999999997</v>
+      </c>
+      <c r="K52"/>
+      <c r="L52" s="5">
+        <f t="shared" si="1"/>
+        <v>34.507199999999997</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A53" s="2">
+        <v>5</v>
+      </c>
+      <c r="B53" s="2">
+        <v>780037001</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="2">
+        <v>12610311174</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F53" s="3">
+        <v>46212</v>
+      </c>
+      <c r="G53" s="2">
+        <v>42.76</v>
+      </c>
+      <c r="H53" s="2">
+        <v>4.2759999999999998</v>
+      </c>
+      <c r="I53" s="2">
+        <v>38.484000000000002</v>
+      </c>
+      <c r="J53" s="5">
+        <f t="shared" si="0"/>
+        <v>35.918399999999991</v>
+      </c>
+      <c r="K53"/>
+      <c r="L53" s="5">
+        <f t="shared" si="1"/>
+        <v>35.918399999999991</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A54" s="2">
+        <v>1</v>
+      </c>
+      <c r="B54" s="2">
+        <v>43000701</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D54" s="2">
+        <v>12610308286</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F54" s="3">
+        <v>46204</v>
+      </c>
+      <c r="G54" s="2">
+        <v>11.76</v>
+      </c>
+      <c r="H54" s="2">
+        <v>1.1759999999999999</v>
+      </c>
+      <c r="I54" s="2">
+        <v>10.584</v>
+      </c>
+      <c r="J54" s="5">
+        <f t="shared" si="0"/>
+        <v>9.8783999999999992</v>
+      </c>
+      <c r="K54"/>
+      <c r="L54" s="5">
+        <f t="shared" si="1"/>
+        <v>9.8783999999999992</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A55" s="2">
+        <v>2</v>
+      </c>
+      <c r="B55" s="2">
+        <v>43001501</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D55" s="2">
+        <v>12610322211</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F55" s="3">
+        <v>46229</v>
+      </c>
+      <c r="G55" s="2">
+        <v>11.17</v>
+      </c>
+      <c r="H55" s="2">
+        <v>1.117</v>
+      </c>
+      <c r="I55" s="2">
+        <v>10.053000000000001</v>
+      </c>
+      <c r="J55" s="5">
+        <f t="shared" si="0"/>
+        <v>9.3827999999999996</v>
+      </c>
+      <c r="K55"/>
+      <c r="L55" s="5">
+        <f t="shared" si="1"/>
+        <v>9.3827999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update claims data - Thu 08/06/2026 20:36:41.65
</commit_message>
<xml_diff>
--- a/الشركة العربية الأوروبية للتأمين.xlsx
+++ b/الشركة العربية الأوروبية للتأمين.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pharmacy_Operations\Insurance_Accounts\Insurance_Claims\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84FA6145-CE80-4A37-B0AC-2D5BD3D6ED0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16247CB6-12D8-4D83-A0A9-330D65D35ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EE0FC3C9-C345-45F5-AA63-81B16FD29943}"/>
   </bookViews>
@@ -207,7 +207,374 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="24">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.000\ _د_._ا_._‏"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.000\ _د_._ا_._‏"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.000\ _د_._ا_._‏"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="9"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.000\ _د_._ا_._‏"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor indexed="17"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.000\ _د_._ا_._‏"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.000\ _د_._ا_._‏"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -218,6 +585,34 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29F9D3A7-A410-4E75-9567-5559742FE035}" name="Table1" displayName="Table1" ref="A1:L56" totalsRowCount="1" headerRowDxfId="12">
+  <autoFilter ref="A1:L55" xr:uid="{29F9D3A7-A410-4E75-9567-5559742FE035}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L55">
+    <sortCondition ref="F1:F55"/>
+  </sortState>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{40336687-55C6-4DBF-B64C-F3C0D9AD1D6D}" name="الرقم" dataDxfId="23" totalsRowDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D061CD9E-2F7E-4528-BE3D-C0505C01813D}" name="رقم الموظف /رقم البطاقة" dataDxfId="22" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{76D9A2AC-27F4-4C84-9F63-F0E2C4A3A429}" name="اسم المريض" dataDxfId="21" totalsRowDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{8EADC87E-806C-44A1-BDDF-ED5BBD572FA0}" name="رقم النموذج" dataDxfId="20" totalsRowDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{8B1C419E-4281-4B4D-A02B-AA98CCA7FE75}" name="نوع المستفيد" dataDxfId="19" totalsRowDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{36A22F97-8B79-40A7-ACD4-67B21B73431D}" name="تاريخ البيع" dataDxfId="18" totalsRowDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{90C2D3E1-AA0A-4D68-94E5-BBF511CE67CA}" name="قيمة الفاتورة" dataDxfId="17" totalsRowDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{B20CFF15-B5E8-4588-88A3-E5249297378F}" name="قيمة المشاركة" dataDxfId="16" totalsRowDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{D791A33F-6B84-4F86-B96D-1983D9944BB3}" name="صافي القيمة" dataDxfId="15" totalsRowDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{7F71AB19-398C-43C4-9365-FBFE695FBEA7}" name="القيمة المطلوبة" totalsRowFunction="sum" dataDxfId="14" totalsRowDxfId="2">
+      <calculatedColumnFormula>G2*0.94-H2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{A3649768-F616-4F61-96AE-8634E5589F1A}" name="المدفوع" totalsRowDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{3D0AE5B1-0491-4F72-A2A6-4B7FFB82F8D3}" name="المتبقي" dataDxfId="13" totalsRowDxfId="0">
+      <calculatedColumnFormula>J2-K2</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -537,17 +932,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD29ECF-A88D-43BD-A0BB-A219CBC2F6D8}">
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.19921875" customWidth="1"/>
+    <col min="2" max="2" width="16.59765625" customWidth="1"/>
     <col min="3" max="3" width="35.296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="9.296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.19921875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.69921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.8984375" customWidth="1"/>
+    <col min="8" max="8" width="10.3984375" customWidth="1"/>
     <col min="9" max="9" width="13.296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.19921875" style="5" customWidth="1"/>
     <col min="11" max="11" width="7.69921875" style="5" bestFit="1" customWidth="1"/>
@@ -658,11 +1053,11 @@
         <v>17.032</v>
       </c>
       <c r="J3" s="5">
-        <f t="shared" ref="J3:J55" si="0">G3*0.94-H3</f>
+        <f>G3*0.94-H3</f>
         <v>15.7546</v>
       </c>
       <c r="L3" s="5">
-        <f t="shared" ref="L3:L55" si="1">J3-K3</f>
+        <f>J3-K3</f>
         <v>15.7546</v>
       </c>
     </row>
@@ -695,11 +1090,11 @@
         <v>26.541</v>
       </c>
       <c r="J4" s="5">
-        <f t="shared" si="0"/>
+        <f>G4*0.94-H4</f>
         <v>24.771599999999999</v>
       </c>
       <c r="L4" s="5">
-        <f t="shared" si="1"/>
+        <f>J4-K4</f>
         <v>24.771599999999999</v>
       </c>
     </row>
@@ -732,11 +1127,11 @@
         <v>19.602</v>
       </c>
       <c r="J5" s="5">
-        <f t="shared" si="0"/>
+        <f>G5*0.94-H5</f>
         <v>18.295199999999998</v>
       </c>
       <c r="L5" s="5">
-        <f t="shared" si="1"/>
+        <f>J5-K5</f>
         <v>18.295199999999998</v>
       </c>
     </row>
@@ -769,11 +1164,11 @@
         <v>27.567</v>
       </c>
       <c r="J6" s="5">
-        <f t="shared" si="0"/>
+        <f>G6*0.94-H6</f>
         <v>25.729199999999999</v>
       </c>
       <c r="L6" s="5">
-        <f t="shared" si="1"/>
+        <f>J6-K6</f>
         <v>25.729199999999999</v>
       </c>
     </row>
@@ -806,11 +1201,11 @@
         <v>32.256</v>
       </c>
       <c r="J7" s="5">
-        <f t="shared" si="0"/>
+        <f>G7*0.94-H7</f>
         <v>30.105599999999999</v>
       </c>
       <c r="L7" s="5">
-        <f t="shared" si="1"/>
+        <f>J7-K7</f>
         <v>30.105599999999999</v>
       </c>
     </row>
@@ -843,11 +1238,11 @@
         <v>34.713000000000001</v>
       </c>
       <c r="J8" s="5">
-        <f t="shared" si="0"/>
+        <f>G8*0.94-H8</f>
         <v>32.398800000000001</v>
       </c>
       <c r="L8" s="5">
-        <f t="shared" si="1"/>
+        <f>J8-K8</f>
         <v>32.398800000000001</v>
       </c>
     </row>
@@ -880,11 +1275,11 @@
         <v>33.920999999999999</v>
       </c>
       <c r="J9" s="5">
-        <f t="shared" si="0"/>
+        <f>G9*0.94-H9</f>
         <v>31.659599999999998</v>
       </c>
       <c r="L9" s="5">
-        <f t="shared" si="1"/>
+        <f>J9-K9</f>
         <v>31.659599999999998</v>
       </c>
     </row>
@@ -917,11 +1312,11 @@
         <v>19.62</v>
       </c>
       <c r="J10" s="5">
-        <f t="shared" si="0"/>
+        <f>G10*0.94-H10</f>
         <v>18.312000000000001</v>
       </c>
       <c r="L10" s="5">
-        <f t="shared" si="1"/>
+        <f>J10-K10</f>
         <v>18.312000000000001</v>
       </c>
     </row>
@@ -954,11 +1349,11 @@
         <v>33.920999999999999</v>
       </c>
       <c r="J11" s="5">
-        <f t="shared" si="0"/>
+        <f>G11*0.94-H11</f>
         <v>31.659599999999998</v>
       </c>
       <c r="L11" s="5">
-        <f t="shared" si="1"/>
+        <f>J11-K11</f>
         <v>31.659599999999998</v>
       </c>
     </row>
@@ -991,11 +1386,11 @@
         <v>40.194000000000003</v>
       </c>
       <c r="J12" s="5">
-        <f t="shared" si="0"/>
+        <f>G12*0.94-H12</f>
         <v>37.514399999999995</v>
       </c>
       <c r="L12" s="5">
-        <f t="shared" si="1"/>
+        <f>J12-K12</f>
         <v>37.514399999999995</v>
       </c>
     </row>
@@ -1028,11 +1423,11 @@
         <v>25.128</v>
       </c>
       <c r="J13" s="5">
-        <f t="shared" si="0"/>
+        <f>G13*0.94-H13</f>
         <v>23.452800000000003</v>
       </c>
       <c r="L13" s="5">
-        <f t="shared" si="1"/>
+        <f>J13-K13</f>
         <v>23.452800000000003</v>
       </c>
     </row>
@@ -1065,11 +1460,11 @@
         <v>29.358000000000001</v>
       </c>
       <c r="J14" s="5">
-        <f t="shared" si="0"/>
+        <f>G14*0.94-H14</f>
         <v>27.400799999999997</v>
       </c>
       <c r="L14" s="5">
-        <f t="shared" si="1"/>
+        <f>J14-K14</f>
         <v>27.400799999999997</v>
       </c>
     </row>
@@ -1102,11 +1497,11 @@
         <v>35.334000000000003</v>
       </c>
       <c r="J15" s="5">
-        <f t="shared" si="0"/>
+        <f>G15*0.94-H15</f>
         <v>32.978399999999993</v>
       </c>
       <c r="L15" s="5">
-        <f t="shared" si="1"/>
+        <f>J15-K15</f>
         <v>32.978399999999993</v>
       </c>
     </row>
@@ -1139,11 +1534,11 @@
         <v>33.920999999999999</v>
       </c>
       <c r="J16" s="5">
-        <f t="shared" si="0"/>
+        <f>G16*0.94-H16</f>
         <v>31.659599999999998</v>
       </c>
       <c r="L16" s="5">
-        <f t="shared" si="1"/>
+        <f>J16-K16</f>
         <v>31.659599999999998</v>
       </c>
     </row>
@@ -1176,11 +1571,11 @@
         <v>40.823999999999998</v>
       </c>
       <c r="J17" s="5">
-        <f t="shared" si="0"/>
+        <f>G17*0.94-H17</f>
         <v>38.102399999999996</v>
       </c>
       <c r="L17" s="5">
-        <f t="shared" si="1"/>
+        <f>J17-K17</f>
         <v>38.102399999999996</v>
       </c>
     </row>
@@ -1213,11 +1608,11 @@
         <v>36.828000000000003</v>
       </c>
       <c r="J18" s="5">
-        <f t="shared" si="0"/>
+        <f>G18*0.94-H18</f>
         <v>34.372799999999998</v>
       </c>
       <c r="L18" s="5">
-        <f t="shared" si="1"/>
+        <f>J18-K18</f>
         <v>34.372799999999998</v>
       </c>
     </row>
@@ -1250,11 +1645,11 @@
         <v>116.09099999999999</v>
       </c>
       <c r="J19" s="5">
-        <f t="shared" si="0"/>
+        <f>G19*0.94-H19</f>
         <v>108.3516</v>
       </c>
       <c r="L19" s="5">
-        <f t="shared" si="1"/>
+        <f>J19-K19</f>
         <v>108.3516</v>
       </c>
     </row>
@@ -1287,11 +1682,11 @@
         <v>33.920999999999999</v>
       </c>
       <c r="J20" s="5">
-        <f t="shared" si="0"/>
+        <f>G20*0.94-H20</f>
         <v>31.659599999999998</v>
       </c>
       <c r="L20" s="5">
-        <f t="shared" si="1"/>
+        <f>J20-K20</f>
         <v>31.659599999999998</v>
       </c>
     </row>
@@ -1324,11 +1719,11 @@
         <v>36.234000000000002</v>
       </c>
       <c r="J21" s="5">
-        <f t="shared" si="0"/>
+        <f>G21*0.94-H21</f>
         <v>33.818399999999997</v>
       </c>
       <c r="L21" s="5">
-        <f t="shared" si="1"/>
+        <f>J21-K21</f>
         <v>33.818399999999997</v>
       </c>
     </row>
@@ -1361,11 +1756,11 @@
         <v>48.16</v>
       </c>
       <c r="J22" s="5">
-        <f t="shared" si="0"/>
+        <f>G22*0.94-H22</f>
         <v>44.548000000000002</v>
       </c>
       <c r="L22" s="5">
-        <f t="shared" si="1"/>
+        <f>J22-K22</f>
         <v>44.548000000000002</v>
       </c>
     </row>
@@ -1398,11 +1793,11 @@
         <v>47.637</v>
       </c>
       <c r="J23" s="5">
-        <f t="shared" si="0"/>
+        <f>G23*0.94-H23</f>
         <v>44.461199999999998</v>
       </c>
       <c r="L23" s="5">
-        <f t="shared" si="1"/>
+        <f>J23-K23</f>
         <v>44.461199999999998</v>
       </c>
     </row>
@@ -1435,69 +1830,70 @@
         <v>37.277999999999999</v>
       </c>
       <c r="J24" s="5">
-        <f t="shared" si="0"/>
+        <f>G24*0.94-H24</f>
         <v>34.7928</v>
       </c>
       <c r="L24" s="5">
-        <f t="shared" si="1"/>
+        <f>J24-K24</f>
         <v>34.7928</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="B25" s="2">
-        <v>7810002702</v>
+        <v>268583</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D25" s="2">
-        <v>13</v>
+        <v>803447696</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F25" s="3">
-        <v>45906</v>
+        <v>45903</v>
       </c>
       <c r="G25" s="2">
-        <v>40.26</v>
+        <v>14.067</v>
       </c>
       <c r="H25" s="2">
-        <v>4.0259999999999998</v>
+        <v>1.407</v>
       </c>
       <c r="I25" s="2">
-        <v>36.234000000000002</v>
+        <v>12.66</v>
       </c>
       <c r="J25" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
-      </c>
+        <f>G25*0.94-H25</f>
+        <v>11.81598</v>
+      </c>
+      <c r="K25"/>
       <c r="L25" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J25-K25</f>
+        <v>11.81598</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="2">
-        <v>780002702</v>
+        <v>7810002702</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D26" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F26" s="3">
-        <v>45937</v>
+        <v>45906</v>
       </c>
       <c r="G26" s="2">
         <v>40.26</v>
@@ -1509,17 +1905,17 @@
         <v>36.234000000000002</v>
       </c>
       <c r="J26" s="5">
-        <f t="shared" si="0"/>
+        <f>G26*0.94-H26</f>
         <v>33.818399999999997</v>
       </c>
       <c r="L26" s="5">
-        <f t="shared" si="1"/>
+        <f>J26-K26</f>
         <v>33.818399999999997</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="2">
         <v>780002702</v>
@@ -1528,13 +1924,13 @@
         <v>8</v>
       </c>
       <c r="D27" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F27" s="3">
-        <v>45970</v>
+        <v>45937</v>
       </c>
       <c r="G27" s="2">
         <v>40.26</v>
@@ -1546,17 +1942,17 @@
         <v>36.234000000000002</v>
       </c>
       <c r="J27" s="5">
-        <f t="shared" si="0"/>
+        <f>G27*0.94-H27</f>
         <v>33.818399999999997</v>
       </c>
       <c r="L27" s="5">
-        <f t="shared" si="1"/>
+        <f>J27-K27</f>
         <v>33.818399999999997</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="2">
         <v>780002702</v>
@@ -1565,13 +1961,13 @@
         <v>8</v>
       </c>
       <c r="D28" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F28" s="3">
-        <v>45999</v>
+        <v>45970</v>
       </c>
       <c r="G28" s="2">
         <v>40.26</v>
@@ -1583,251 +1979,251 @@
         <v>36.234000000000002</v>
       </c>
       <c r="J28" s="5">
-        <f t="shared" si="0"/>
+        <f>G28*0.94-H28</f>
         <v>33.818399999999997</v>
       </c>
       <c r="L28" s="5">
-        <f t="shared" si="1"/>
+        <f>J28-K28</f>
         <v>33.818399999999997</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="2">
-        <v>780037001</v>
+        <v>780002702</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D29" s="2">
-        <v>12510189537</v>
+        <v>16</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F29" s="3">
-        <v>46009</v>
+        <v>45999</v>
       </c>
       <c r="G29" s="2">
-        <v>20.89</v>
+        <v>40.26</v>
       </c>
       <c r="H29" s="2">
-        <v>2.089</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I29" s="2">
-        <v>18.800999999999998</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J29" s="5">
-        <f t="shared" si="0"/>
-        <v>17.547599999999999</v>
+        <f>G29*0.94-H29</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="L29" s="5">
-        <f t="shared" si="1"/>
-        <v>17.547599999999999</v>
+        <f>J29-K29</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="2">
-        <v>9841047081</v>
+        <v>780037001</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D30" s="2">
-        <v>12610199442</v>
+        <v>12510189537</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F30" s="3">
-        <v>46023</v>
+        <v>46009</v>
       </c>
       <c r="G30" s="2">
-        <v>68.83</v>
+        <v>20.89</v>
       </c>
       <c r="H30" s="2">
-        <v>0</v>
+        <v>2.089</v>
       </c>
       <c r="I30" s="2">
-        <v>68.83</v>
+        <v>18.800999999999998</v>
       </c>
       <c r="J30" s="5">
-        <f t="shared" si="0"/>
-        <v>64.700199999999995</v>
+        <f>G30*0.94-H30</f>
+        <v>17.547599999999999</v>
       </c>
       <c r="L30" s="5">
-        <f t="shared" si="1"/>
-        <v>64.700199999999995</v>
+        <f>J30-K30</f>
+        <v>17.547599999999999</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="2">
-        <v>780002702</v>
+        <v>9841047081</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D31" s="2">
-        <v>17</v>
+        <v>12610199442</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F31" s="3">
-        <v>46026</v>
+        <v>46023</v>
       </c>
       <c r="G31" s="2">
-        <v>40.26</v>
+        <v>68.83</v>
       </c>
       <c r="H31" s="2">
-        <v>4.0259999999999998</v>
+        <v>0</v>
       </c>
       <c r="I31" s="2">
-        <v>36.234000000000002</v>
+        <v>68.83</v>
       </c>
       <c r="J31" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G31*0.94-H31</f>
+        <v>64.700199999999995</v>
       </c>
       <c r="L31" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J31-K31</f>
+        <v>64.700199999999995</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" s="2">
-        <v>780037001</v>
+        <v>780002702</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D32" s="2">
-        <v>12610202650</v>
+        <v>17</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F32" s="3">
-        <v>46032</v>
+        <v>46026</v>
       </c>
       <c r="G32" s="2">
-        <v>15.93</v>
+        <v>40.26</v>
       </c>
       <c r="H32" s="2">
-        <v>1.593</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I32" s="2">
-        <v>14.337</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J32" s="5">
-        <f t="shared" si="0"/>
-        <v>13.3812</v>
+        <f>G32*0.94-H32</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="L32" s="5">
-        <f t="shared" si="1"/>
-        <v>13.3812</v>
+        <f>J32-K32</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="2">
-        <v>780002702</v>
+        <v>780037001</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D33" s="2">
-        <v>18</v>
+        <v>12610202650</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F33" s="3">
-        <v>46062</v>
+        <v>46032</v>
       </c>
       <c r="G33" s="2">
-        <v>40.26</v>
+        <v>15.93</v>
       </c>
       <c r="H33" s="2">
-        <v>4.0259999999999998</v>
+        <v>1.593</v>
       </c>
       <c r="I33" s="2">
-        <v>36.234000000000002</v>
+        <v>14.337</v>
       </c>
       <c r="J33" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G33*0.94-H33</f>
+        <v>13.3812</v>
       </c>
       <c r="L33" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J33-K33</f>
+        <v>13.3812</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="2">
-        <v>780037004</v>
+        <v>780002702</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D34" s="2">
-        <v>12610223377</v>
+        <v>18</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F34" s="3">
-        <v>46066</v>
+        <v>46062</v>
       </c>
       <c r="G34" s="2">
-        <v>39.950000000000003</v>
+        <v>40.26</v>
       </c>
       <c r="H34" s="2">
-        <v>3.9950000000000001</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I34" s="2">
-        <v>35.954999999999998</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J34" s="5">
-        <f t="shared" si="0"/>
-        <v>33.558</v>
+        <f>G34*0.94-H34</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="L34" s="5">
-        <f t="shared" si="1"/>
-        <v>33.558</v>
+        <f>J34-K34</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="2">
-        <v>780037001</v>
+        <v>780037004</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D35" s="2">
-        <v>12610223361</v>
+        <v>12610223377</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F35" s="3">
         <v>46066</v>
@@ -1842,54 +2238,54 @@
         <v>35.954999999999998</v>
       </c>
       <c r="J35" s="5">
-        <f t="shared" si="0"/>
+        <f>G35*0.94-H35</f>
         <v>33.558</v>
       </c>
       <c r="L35" s="5">
-        <f t="shared" si="1"/>
+        <f>J35-K35</f>
         <v>33.558</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>780002702</v>
+        <v>780037001</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D36" s="2">
-        <v>19</v>
+        <v>12610223361</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F36" s="3">
-        <v>46112</v>
+        <v>46066</v>
       </c>
       <c r="G36" s="2">
-        <v>40.26</v>
+        <v>39.950000000000003</v>
       </c>
       <c r="H36" s="2">
-        <v>4.0259999999999998</v>
+        <v>3.9950000000000001</v>
       </c>
       <c r="I36" s="2">
-        <v>36.234000000000002</v>
+        <v>35.954999999999998</v>
       </c>
       <c r="J36" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G36*0.94-H36</f>
+        <v>33.558</v>
       </c>
       <c r="L36" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J36-K36</f>
+        <v>33.558</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="B37" s="2">
         <v>780002702</v>
@@ -1916,431 +2312,430 @@
         <v>36.234000000000002</v>
       </c>
       <c r="J37" s="5">
-        <f t="shared" si="0"/>
+        <f>G37*0.94-H37</f>
         <v>33.818399999999997</v>
       </c>
-      <c r="K37"/>
       <c r="L37" s="5">
-        <f t="shared" si="1"/>
+        <f>J37-K37</f>
         <v>33.818399999999997</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B38" s="2">
-        <v>950001201</v>
+        <v>780002702</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D38" s="2">
-        <v>12610254681</v>
+        <v>19</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F38" s="3">
-        <v>46118</v>
+        <v>46112</v>
       </c>
       <c r="G38" s="2">
-        <v>43.98</v>
+        <v>40.26</v>
       </c>
       <c r="H38" s="2">
-        <v>10.994999999999999</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I38" s="2">
-        <v>32.984999999999999</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J38" s="5">
-        <f t="shared" si="0"/>
-        <v>30.346199999999996</v>
+        <f>G38*0.94-H38</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="K38"/>
       <c r="L38" s="5">
-        <f t="shared" si="1"/>
-        <v>30.346199999999996</v>
+        <f>J38-K38</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B39" s="2">
-        <v>950006601</v>
+        <v>950001201</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D39" s="2">
-        <v>12610256118</v>
+        <v>12610254681</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F39" s="3">
-        <v>46120</v>
+        <v>46118</v>
       </c>
       <c r="G39" s="2">
-        <v>25.45</v>
+        <v>43.98</v>
       </c>
       <c r="H39" s="2">
-        <v>6.3620000000000001</v>
+        <v>10.994999999999999</v>
       </c>
       <c r="I39" s="2">
-        <v>19.088000000000001</v>
+        <v>32.984999999999999</v>
       </c>
       <c r="J39" s="5">
-        <f t="shared" si="0"/>
-        <v>17.561</v>
+        <f>G39*0.94-H39</f>
+        <v>30.346199999999996</v>
       </c>
       <c r="K39"/>
       <c r="L39" s="5">
-        <f t="shared" si="1"/>
-        <v>17.561</v>
+        <f>J39-K39</f>
+        <v>30.346199999999996</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B40" s="2">
-        <v>780002702</v>
+        <v>950006601</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="D40" s="2">
-        <v>20</v>
+        <v>12610256118</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F40" s="3">
-        <v>46121</v>
+        <v>46120</v>
       </c>
       <c r="G40" s="2">
-        <v>40.26</v>
+        <v>25.45</v>
       </c>
       <c r="H40" s="2">
-        <v>4.0259999999999998</v>
+        <v>6.3620000000000001</v>
       </c>
       <c r="I40" s="2">
-        <v>36.234000000000002</v>
+        <v>19.088000000000001</v>
       </c>
       <c r="J40" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G40*0.94-H40</f>
+        <v>17.561</v>
       </c>
       <c r="K40"/>
       <c r="L40" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J40-K40</f>
+        <v>17.561</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B41" s="2">
-        <v>780037001</v>
+        <v>780002702</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D41" s="2">
-        <v>12610257018</v>
+        <v>20</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F41" s="3">
-        <v>46126</v>
+        <v>46121</v>
       </c>
       <c r="G41" s="2">
-        <v>6.35</v>
+        <v>40.26</v>
       </c>
       <c r="H41" s="2">
-        <v>0.63500000000000001</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I41" s="2">
-        <v>5.7149999999999999</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J41" s="5">
-        <f t="shared" si="0"/>
-        <v>5.3339999999999996</v>
+        <f>G41*0.94-H41</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="K41"/>
       <c r="L41" s="5">
-        <f t="shared" si="1"/>
-        <v>5.3339999999999996</v>
+        <f>J41-K41</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B42" s="2">
-        <v>780037004</v>
+        <v>780037001</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D42" s="2">
-        <v>12610257015</v>
+        <v>12610257018</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F42" s="3">
         <v>46126</v>
       </c>
       <c r="G42" s="2">
-        <v>31.98</v>
+        <v>6.35</v>
       </c>
       <c r="H42" s="2">
-        <v>3.198</v>
+        <v>0.63500000000000001</v>
       </c>
       <c r="I42" s="2">
-        <v>28.782</v>
+        <v>5.7149999999999999</v>
       </c>
       <c r="J42" s="5">
-        <f t="shared" si="0"/>
-        <v>26.863199999999999</v>
+        <f>G42*0.94-H42</f>
+        <v>5.3339999999999996</v>
       </c>
       <c r="K42"/>
       <c r="L42" s="5">
-        <f t="shared" si="1"/>
-        <v>26.863199999999999</v>
+        <f>J42-K42</f>
+        <v>5.3339999999999996</v>
       </c>
     </row>
     <row r="43" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B43" s="2">
-        <v>780002702</v>
+        <v>780037004</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D43" s="2">
-        <v>21</v>
+        <v>12610257015</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F43" s="3">
-        <v>46153</v>
+        <v>46126</v>
       </c>
       <c r="G43" s="2">
-        <v>40.26</v>
+        <v>31.98</v>
       </c>
       <c r="H43" s="2">
-        <v>4.0259999999999998</v>
+        <v>3.198</v>
       </c>
       <c r="I43" s="2">
-        <v>36.234000000000002</v>
+        <v>28.782</v>
       </c>
       <c r="J43" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G43*0.94-H43</f>
+        <v>26.863199999999999</v>
       </c>
       <c r="K43"/>
       <c r="L43" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J43-K43</f>
+        <v>26.863199999999999</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B44" s="2">
-        <v>780002702</v>
+        <v>62004401</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D44" s="2">
-        <v>22</v>
+        <v>12610269342</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F44" s="3">
-        <v>46178</v>
+        <v>46140</v>
       </c>
       <c r="G44" s="2">
-        <v>40.26</v>
+        <v>12.5</v>
       </c>
       <c r="H44" s="2">
-        <v>4.0259999999999998</v>
+        <v>1.925</v>
       </c>
       <c r="I44" s="2">
-        <v>36.234000000000002</v>
+        <v>10.574999999999999</v>
       </c>
       <c r="J44" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G44*0.94-H44</f>
+        <v>9.8249999999999993</v>
       </c>
       <c r="K44"/>
       <c r="L44" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J44-K44</f>
+        <v>9.8249999999999993</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B45" s="2">
-        <v>268583</v>
+        <v>780002702</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D45" s="2">
-        <v>803447696</v>
+        <v>21</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F45" s="3">
-        <v>45903</v>
+        <v>46153</v>
       </c>
       <c r="G45" s="2">
-        <v>14.067</v>
+        <v>40.26</v>
       </c>
       <c r="H45" s="2">
-        <v>1.407</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I45" s="2">
-        <v>12.66</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J45" s="5">
-        <f t="shared" si="0"/>
-        <v>11.81598</v>
+        <f>G45*0.94-H45</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="K45"/>
       <c r="L45" s="5">
-        <f t="shared" si="1"/>
-        <v>11.81598</v>
+        <f>J45-K45</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B46" s="2">
-        <v>62004401</v>
+        <v>43001502</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D46" s="2">
-        <v>12610269342</v>
+        <v>12610285384</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F46" s="3">
-        <v>46140</v>
+        <v>46164</v>
       </c>
       <c r="G46" s="2">
         <v>12.5</v>
       </c>
       <c r="H46" s="2">
-        <v>1.925</v>
+        <v>1.25</v>
       </c>
       <c r="I46" s="2">
-        <v>10.574999999999999</v>
+        <v>11.25</v>
       </c>
       <c r="J46" s="5">
-        <f t="shared" si="0"/>
-        <v>9.8249999999999993</v>
+        <f>G46*0.94-H46</f>
+        <v>10.5</v>
       </c>
       <c r="K46"/>
       <c r="L46" s="5">
-        <f t="shared" si="1"/>
-        <v>9.8249999999999993</v>
+        <f>J46-K46</f>
+        <v>10.5</v>
       </c>
     </row>
     <row r="47" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B47" s="2">
-        <v>43001502</v>
+        <v>50016401</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D47" s="2">
-        <v>12610285384</v>
+        <v>12610292185</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F47" s="3">
-        <v>46164</v>
+        <v>46177</v>
       </c>
       <c r="G47" s="2">
         <v>12.5</v>
       </c>
       <c r="H47" s="2">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c r="I47" s="2">
-        <v>11.25</v>
+        <v>10</v>
       </c>
       <c r="J47" s="5">
-        <f t="shared" si="0"/>
-        <v>10.5</v>
+        <f>G47*0.94-H47</f>
+        <v>9.25</v>
       </c>
       <c r="K47"/>
       <c r="L47" s="5">
-        <f t="shared" si="1"/>
-        <v>10.5</v>
+        <f>J47-K47</f>
+        <v>9.25</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B48" s="2">
-        <v>50016401</v>
+        <v>780002702</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="D48" s="2">
-        <v>12610292185</v>
+        <v>22</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F48" s="3">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="G48" s="2">
-        <v>12.5</v>
+        <v>40.26</v>
       </c>
       <c r="H48" s="2">
-        <v>2.5</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I48" s="2">
-        <v>10</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J48" s="5">
-        <f t="shared" si="0"/>
-        <v>9.25</v>
+        <f>G48*0.94-H48</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="K48"/>
       <c r="L48" s="5">
-        <f t="shared" si="1"/>
-        <v>9.25</v>
+        <f>J48-K48</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="49" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
@@ -2348,51 +2743,51 @@
         <v>1</v>
       </c>
       <c r="B49" s="2">
-        <v>780037005</v>
+        <v>43000701</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D49" s="2">
-        <v>12610309392</v>
+        <v>12610308286</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F49" s="3">
-        <v>46207</v>
+        <v>46204</v>
       </c>
       <c r="G49" s="2">
-        <v>44.66</v>
+        <v>11.76</v>
       </c>
       <c r="H49" s="2">
-        <v>4.4660000000000002</v>
+        <v>1.1759999999999999</v>
       </c>
       <c r="I49" s="2">
-        <v>40.194000000000003</v>
+        <v>10.584</v>
       </c>
       <c r="J49" s="5">
-        <f t="shared" si="0"/>
-        <v>37.514399999999995</v>
+        <f>G49*0.94-H49</f>
+        <v>9.8783999999999992</v>
       </c>
       <c r="K49"/>
       <c r="L49" s="5">
-        <f t="shared" si="1"/>
-        <v>37.514399999999995</v>
+        <f>J49-K49</f>
+        <v>9.8783999999999992</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B50" s="2">
-        <v>780037003</v>
+        <v>780037005</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D50" s="2">
-        <v>12610309395</v>
+        <v>12610309392</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>12</v>
@@ -2401,174 +2796,174 @@
         <v>46207</v>
       </c>
       <c r="G50" s="2">
-        <v>54.41</v>
+        <v>44.66</v>
       </c>
       <c r="H50" s="2">
-        <v>5.4409999999999998</v>
+        <v>4.4660000000000002</v>
       </c>
       <c r="I50" s="2">
-        <v>48.969000000000001</v>
+        <v>40.194000000000003</v>
       </c>
       <c r="J50" s="5">
-        <f t="shared" si="0"/>
-        <v>45.704399999999993</v>
+        <f>G50*0.94-H50</f>
+        <v>37.514399999999995</v>
       </c>
       <c r="K50"/>
       <c r="L50" s="5">
-        <f t="shared" si="1"/>
-        <v>45.704399999999993</v>
+        <f>J50-K50</f>
+        <v>37.514399999999995</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B51" s="2">
-        <v>780002702</v>
+        <v>780037003</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D51" s="2">
-        <v>23</v>
+        <v>12610309395</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F51" s="3">
-        <v>46209</v>
+        <v>46207</v>
       </c>
       <c r="G51" s="2">
-        <v>40.26</v>
+        <v>54.41</v>
       </c>
       <c r="H51" s="2">
-        <v>4.0259999999999998</v>
+        <v>5.4409999999999998</v>
       </c>
       <c r="I51" s="2">
-        <v>36.234000000000002</v>
+        <v>48.969000000000001</v>
       </c>
       <c r="J51" s="5">
-        <f t="shared" si="0"/>
-        <v>33.818399999999997</v>
+        <f>G51*0.94-H51</f>
+        <v>45.704399999999993</v>
       </c>
       <c r="K51"/>
       <c r="L51" s="5">
-        <f t="shared" si="1"/>
-        <v>33.818399999999997</v>
+        <f>J51-K51</f>
+        <v>45.704399999999993</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B52" s="2">
-        <v>780037004</v>
+        <v>780002702</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="D52" s="2">
-        <v>12610311180</v>
+        <v>23</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F52" s="3">
-        <v>46212</v>
+        <v>46209</v>
       </c>
       <c r="G52" s="2">
-        <v>41.08</v>
+        <v>40.26</v>
       </c>
       <c r="H52" s="2">
-        <v>4.1079999999999997</v>
+        <v>4.0259999999999998</v>
       </c>
       <c r="I52" s="2">
-        <v>36.972000000000001</v>
+        <v>36.234000000000002</v>
       </c>
       <c r="J52" s="5">
-        <f t="shared" si="0"/>
-        <v>34.507199999999997</v>
+        <f>G52*0.94-H52</f>
+        <v>33.818399999999997</v>
       </c>
       <c r="K52"/>
       <c r="L52" s="5">
-        <f t="shared" si="1"/>
-        <v>34.507199999999997</v>
+        <f>J52-K52</f>
+        <v>33.818399999999997</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" s="2">
-        <v>780037001</v>
+        <v>780037004</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D53" s="2">
-        <v>12610311174</v>
+        <v>12610311180</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F53" s="3">
         <v>46212</v>
       </c>
       <c r="G53" s="2">
-        <v>42.76</v>
+        <v>41.08</v>
       </c>
       <c r="H53" s="2">
-        <v>4.2759999999999998</v>
+        <v>4.1079999999999997</v>
       </c>
       <c r="I53" s="2">
-        <v>38.484000000000002</v>
+        <v>36.972000000000001</v>
       </c>
       <c r="J53" s="5">
-        <f t="shared" si="0"/>
-        <v>35.918399999999991</v>
+        <f>G53*0.94-H53</f>
+        <v>34.507199999999997</v>
       </c>
       <c r="K53"/>
       <c r="L53" s="5">
-        <f t="shared" si="1"/>
-        <v>35.918399999999991</v>
+        <f>J53-K53</f>
+        <v>34.507199999999997</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B54" s="2">
-        <v>43000701</v>
+        <v>780037001</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="D54" s="2">
-        <v>12610308286</v>
+        <v>12610311174</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F54" s="3">
-        <v>46204</v>
+        <v>46212</v>
       </c>
       <c r="G54" s="2">
-        <v>11.76</v>
+        <v>42.76</v>
       </c>
       <c r="H54" s="2">
-        <v>1.1759999999999999</v>
+        <v>4.2759999999999998</v>
       </c>
       <c r="I54" s="2">
-        <v>10.584</v>
+        <v>38.484000000000002</v>
       </c>
       <c r="J54" s="5">
-        <f t="shared" si="0"/>
-        <v>9.8783999999999992</v>
+        <f>G54*0.94-H54</f>
+        <v>35.918399999999991</v>
       </c>
       <c r="K54"/>
       <c r="L54" s="5">
-        <f t="shared" si="1"/>
-        <v>9.8783999999999992</v>
+        <f>J54-K54</f>
+        <v>35.918399999999991</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
@@ -2600,16 +2995,34 @@
         <v>10.053000000000001</v>
       </c>
       <c r="J55" s="5">
-        <f t="shared" si="0"/>
+        <f>G55*0.94-H55</f>
         <v>9.3827999999999996</v>
       </c>
       <c r="K55"/>
       <c r="L55" s="5">
-        <f t="shared" si="1"/>
+        <f>J55-K55</f>
         <v>9.3827999999999996</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="5">
+        <f>SUBTOTAL(109,Table1[القيمة المطلوبة])</f>
+        <v>1646.4253800000004</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>